<commit_message>
Rilascio e pubblicazione rev 1.2
</commit_message>
<xml_diff>
--- a/Indice versioni.xlsx
+++ b/Indice versioni.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gessica.dilenardo\Documents\Power BI\Elaborati\BI_Commerciali\BI_fatturati_commerciale_italia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EC2281-0A3B-4DEE-A24E-4A991534B596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABDA8EE9-313C-4E29-9015-6B216361E4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{E8661EE8-0424-44C1-8E9C-476E929CF0A3}"/>
   </bookViews>
@@ -540,6 +540,9 @@
       <c r="C6" s="1">
         <v>45761</v>
       </c>
+      <c r="D6" s="1">
+        <v>45761</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Creata rev 1.3 per modifiche mail richiesta Marco Alpi 14-04-2025
</commit_message>
<xml_diff>
--- a/Indice versioni.xlsx
+++ b/Indice versioni.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gessica.dilenardo\Documents\Power BI\Elaborati\BI_Commerciali\BI_fatturati_commerciale_italia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABDA8EE9-313C-4E29-9015-6B216361E4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14625305-2C97-441F-8768-67D3F78D747F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{E8661EE8-0424-44C1-8E9C-476E929CF0A3}"/>
+    <workbookView xWindow="-28920" yWindow="-270" windowWidth="29040" windowHeight="15720" xr2:uid="{E8661EE8-0424-44C1-8E9C-476E929CF0A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>n° versione</t>
   </si>
@@ -76,6 +76,12 @@
   </si>
   <si>
     <t>Richiesta mail 30/01/2025 - Copia pagina lettini per diverse categorie (Reck, Struzzo, HandiMove, Tecnologie)</t>
+  </si>
+  <si>
+    <t>1.3</t>
+  </si>
+  <si>
+    <t>Aggiunti elementi al filtro pagina struzzo, come da mail 14/04/2025</t>
   </si>
 </sst>
 </file>
@@ -142,8 +148,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3DA6D639-3982-49E4-9273-EDF18E8E0296}" name="Indice_versioni" displayName="Indice_versioni" ref="A1:D6" totalsRowShown="0">
-  <autoFilter ref="A1:D6" xr:uid="{3DA6D639-3982-49E4-9273-EDF18E8E0296}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3DA6D639-3982-49E4-9273-EDF18E8E0296}" name="Indice_versioni" displayName="Indice_versioni" ref="A1:D7" totalsRowShown="0">
+  <autoFilter ref="A1:D7" xr:uid="{3DA6D639-3982-49E4-9273-EDF18E8E0296}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DF868F52-5EA1-4396-A148-08152EED9F75}" name="n° versione"/>
     <tableColumn id="2" xr3:uid="{4C524CEA-5424-4979-BFA7-A9FA81F03901}" name="Modifiche" dataDxfId="1"/>
@@ -451,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84F82909-EF29-41C9-80BE-D5671978DDB6}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
@@ -544,6 +550,17 @@
         <v>45761</v>
       </c>
     </row>
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="1">
+        <v>45761</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Completata nodifica rev 1.3 e pubblicazione
</commit_message>
<xml_diff>
--- a/Indice versioni.xlsx
+++ b/Indice versioni.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gessica.dilenardo\Documents\Power BI\Elaborati\BI_Commerciali\BI_fatturati_commerciale_italia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14625305-2C97-441F-8768-67D3F78D747F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6539E961-753B-4FC5-A80E-153B0AE81255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-270" windowWidth="29040" windowHeight="15720" xr2:uid="{E8661EE8-0424-44C1-8E9C-476E929CF0A3}"/>
   </bookViews>
@@ -560,6 +560,9 @@
       <c r="C7" s="1">
         <v>45761</v>
       </c>
+      <c r="D7" s="1">
+        <v>45761</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>